<commit_message>
scan: seg7 2026-09-28 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq8_2026-09-24.xlsx
@@ -555,7 +555,7 @@
         <v>70.82555094500356</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>42.70699604767094</v>
+        <v>42.70699612569278</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>3.50021136580328</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.5947603030738264</v>
+        <v>0.5947603028677833</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>65.73815824084545</v>
+        <v>65.73815825712292</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>36.16735080254034</v>
+        <v>36.16735081109153</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.32951480466362</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2.237048119299912</v>
+        <v>2.237048119093824</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,7 +658,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>88.12036762660121</v>
+        <v>88.12036762146396</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>52.76802222817642</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>9.703150061883775</v>
+        <v>9.703150062089811</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>80.59606977886649</v>
+        <v>80.59606979049521</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>38.51526499451232</v>
+        <v>38.51526497614011</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.79021669540324</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>7.700386973471186</v>
+        <v>7.700386973265122</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>84.64618586176012</v>
+        <v>84.64618590643579</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>28.18194124558112</v>
+        <v>28.18194124558111</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.964987880141097</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>5.65552983712274</v>
+        <v>5.655529836690024</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>925.7345786062576</v>
+        <v>925.7345786062572</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>543</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>60.24136509386689</v>
+        <v>60.24136511461965</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>29.89846456184232</v>
+        <v>29.89846454114974</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.7287850130249796</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.9773198892399472</v>
+        <v>0.9773198893429544</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>899.5218934225097</v>
+        <v>899.5218934225098</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>212</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61.56154340923592</v>
+        <v>61.56154340515053</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>20.6013875390675</v>
+        <v>20.60138748824996</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.646130978574432</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1.582751405771736</v>
+        <v>1.582751406080825</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>71.15612114758318</v>
+        <v>71.15612114256673</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>27.96381740672689</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>9.354177174746738</v>
+        <v>9.354177174787958</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -979,7 +979,7 @@
         <v>61.89811437501302</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>24.34335074706336</v>
+        <v>24.34335075024725</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.8722209081356974</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.463588909976806</v>
+        <v>1.463588909667718</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>74.94937897252854</v>
+        <v>74.94937908256603</v>
       </c>
       <c r="I11" s="2" t="n">
         <v>15.7037568089477</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.9119300787667448</v>
+        <v>0.9119300801061192</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         <v>61.23935037709227</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>21.13146529911165</v>
+        <v>21.13146529911164</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.656645262341546</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>4.134038479660652</v>
+        <v>4.134038478836409</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>73.4003942527995</v>
+        <v>73.40039407334228</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>24.66302365221904</v>
+        <v>24.66302370393021</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>6.896318692442442</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.47615805895507</v>
+        <v>1.476158059470213</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.20963151049805</v>
+        <v>60.20963148408136</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>19.50827042380282</v>
+        <v>19.50827034222214</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.96418142760855</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>5.155443504174425</v>
+        <v>5.155443507059225</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>785.9471804295572</v>
+        <v>785.9471804295571</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>760</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>60.57119885505033</v>
+        <v>60.57119890552397</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>19.74367256331789</v>
+        <v>19.74367257648731</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.464175916175535</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>10.06426793804138</v>
+        <v>10.06426793670204</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>766.2575404143543</v>
+        <v>766.2575404143539</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>31.15</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>71.99656052416603</v>
+        <v>71.99656052948484</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>61.58538771716989</v>
+        <v>61.5853877572023</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.151407788814635</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.3573129381493694</v>
+        <v>0.3573129383142135</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>765.942760757848</v>
+        <v>765.9427607578477</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>920</v>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57.41107419165718</v>
+        <v>57.41107416965205</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>11.03507967330474</v>
+        <v>11.03507969234604</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.928030176784718</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>5.26607900575506</v>
+        <v>5.266079005445951</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>736.2092007540347</v>
+        <v>736.2092007540349</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>162.5</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>60.96365504767504</v>
+        <v>60.96365472454443</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>16.05187961152815</v>
+        <v>16.05187964734687</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.95934996305407</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.405953837981309</v>
+        <v>1.405953840474611</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>63.90508958635206</v>
+        <v>63.90508980610159</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>17.65705384779894</v>
+        <v>17.65705385881593</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.026247695877518</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>5.059281735524316</v>
+        <v>5.059281732021321</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,7 +1506,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>58.69253905590983</v>
+        <v>58.6925391057643</v>
       </c>
       <c r="I20" s="2" t="n">
         <v>25.26471035215904</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.956713710893764</v>
+        <v>0.9567137103786276</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>59.49033411790953</v>
+        <v>59.49033415846048</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>21.08751461848973</v>
+        <v>21.08751463240392</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.131605854810355</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.265345980032246</v>
+        <v>1.265345980238305</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>66.16320059898726</v>
+        <v>66.16320063894881</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>40.57215952288742</v>
+        <v>40.57215948541117</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.4749616713588787</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.3246504555247913</v>
+        <v>0.3246504560811498</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>659.3675222157659</v>
+        <v>659.367522215766</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>203</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>56.69909797316673</v>
+        <v>56.699097918556</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>36.68749386734824</v>
+        <v>36.68749386794412</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.4801528806772076</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.0943347645978414</v>
+        <v>0.0943347645566244</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>647.852052627091</v>
+        <v>647.8520526270894</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>26</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>61.46742358312015</v>
+        <v>61.46742347205804</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>26.82029575405285</v>
+        <v>26.82029584265646</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.9874025605664936</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>65.13566853230236</v>
+        <v>65.13566849947772</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>40.19505526253655</v>
+        <v>40.19505521140578</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>2.095972335302705</v>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>638.5851997171108</v>
+        <v>638.5851997171106</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>241</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>60.68122755006476</v>
+        <v>60.68122759345317</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>36.96136074814684</v>
+        <v>36.96136082243196</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.3678965103766107</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.836592912394379</v>
+        <v>1.836592911570146</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>63.58352309851157</v>
+        <v>63.58352312051476</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>27.89889848691482</v>
+        <v>27.89889847429074</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>3.23943968405878</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.2018402120506409</v>
+        <v>0.201840212163972</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>621.7126840857225</v>
+        <v>621.7126840857229</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>367</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>58.6470030670588</v>
+        <v>58.64700291271885</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>28.68549038317942</v>
+        <v>28.68549034526885</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.6132911845246226</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.548265761157396</v>
+        <v>1.548265763423979</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>617.5235908407381</v>
+        <v>617.5235908407383</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>121</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>59.77957890163655</v>
+        <v>59.77957896588754</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>39.21054991730875</v>
+        <v>39.21054989516679</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.6433430915393756</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1882100985569996</v>
+        <v>0.1882100983509431</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>616.5411665595871</v>
+        <v>616.5411665595872</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>222.5</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>54.8741790117131</v>
+        <v>54.87417903911388</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>31.7410701216534</v>
+        <v>31.74107012414833</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.778876730455374</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.1176190992164976</v>
+        <v>0.1176190998346982</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>609.7976409574533</v>
+        <v>609.7976409574532</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>2750</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>49.02213548488023</v>
+        <v>49.02213551717188</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>17.63059830228329</v>
+        <v>17.63059829913762</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.8553368734082714</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>11.04519937633098</v>
+        <v>11.04519937159101</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>58.28766713946622</v>
+        <v>58.28766715545677</v>
       </c>
       <c r="I34" s="2" t="n">
         <v>34.23908860829906</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.2091429648280574</v>
+        <v>0.2091429646426021</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>55.94041245730718</v>
+        <v>55.94041261046966</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>26.19077986526846</v>
+        <v>26.19077985797317</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.4460736239295284</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-1.094568679457769</v>
+        <v>-1.09456867925168</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>564.6153494509051</v>
+        <v>564.615349450905</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>83</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>55.90906285961826</v>
+        <v>55.90906283543966</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>42.23952001010795</v>
+        <v>42.23952009668248</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.3749508866699448</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.1814221267022195</v>
+        <v>-0.1814221264961595</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>51.58661034954125</v>
+        <v>51.58661034996177</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>15.31131549509424</v>
+        <v>15.31131549178912</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.5051365967127892</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-9.686543584254435</v>
+        <v>-9.686543585903079</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>545.6144112174717</v>
+        <v>545.6144112174882</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>122.5</v>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>55.46447630903453</v>
+        <v>55.46447632677341</v>
       </c>
       <c r="I39" s="2" t="n">
         <v>17.26019775199913</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>1.588952145453673</v>
+        <v>1.588952145082768</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>48.46117474335521</v>
+        <v>48.46117473868623</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>21.13086285145022</v>
+        <v>21.13086286632531</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.3571932736127358</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-1.045889276702913</v>
+        <v>-1.04588927637321</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>51.15670335670375</v>
+        <v>51.15670335808578</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>13.99411228193961</v>
+        <v>13.99411225358634</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.577488279054458</v>
@@ -2672,7 +2672,7 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>53.82603797753615</v>
+        <v>53.82603798567551</v>
       </c>
       <c r="I42" s="2" t="n">
         <v>25.40657876632234</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-3.766801085504554</v>
+        <v>-3.766801086328769</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>43.11358497883407</v>
+        <v>43.11357763512334</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>35.78384473975631</v>
+        <v>35.78384472633256</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1.506827072108643</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0196544874416038</v>
+        <v>0.0196544880597784</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>1.856836412115425</v>
+        <v>1.856836412218478</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>59.10791666461599</v>
+        <v>59.10791685129321</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>20.90060714984936</v>
+        <v>20.90060718451973</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.8831122832831965</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.762619515624255</v>
+        <v>0.7626195154181873</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>49.85256256879666</v>
+        <v>49.85256269669333</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>10.04010459997156</v>
+        <v>10.04010459683971</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.3491499896645576</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.1252319418917889</v>
+        <v>0.1252319418196713</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>443.6981343374557</v>
+        <v>443.698134337455</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>5670</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>40.19284420383227</v>
+        <v>40.192844213586</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>11.65234403940162</v>
+        <v>11.65234407452498</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>1.24083915740281</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-52.74734769584321</v>
+        <v>-52.74734770305497</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>56.78614122979565</v>
+        <v>56.78614114756991</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>23.14120942373325</v>
+        <v>23.1412094684832</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.9701417725852</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0726799342634184</v>
+        <v>0.072679934387053</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>435.1380384103795</v>
+        <v>435.1380384103796</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>17.3</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>45.55765953953925</v>
+        <v>45.55765966704588</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>25.97607906910385</v>
+        <v>25.97607906387721</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6506872437906921</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.015712862087162</v>
+        <v>0.0157128620253457</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
         <v>53.05379800273698</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>18.68221079474088</v>
+        <v>18.68221079673399</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.068079424069768</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.0330769176218203</v>
+        <v>-0.033076917601218</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>47.63819293202531</v>
+        <v>47.6381929455761</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>11.54075634699438</v>
+        <v>11.54075631245025</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.6138697630524275</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.5955569774678642</v>
+        <v>0.5955569773648346</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>427.5302103844984</v>
+        <v>427.5302103844983</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>98</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>51.28007070201726</v>
+        <v>51.28007099387669</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.66629194713751</v>
+        <v>18.66629194508466</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.1007261379169665</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.5991054025063498</v>
+        <v>-0.5991054042578497</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3417,7 +3417,7 @@
         <v>51.65881442467627</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>7.417386015169574</v>
+        <v>7.417385959696069</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.2942788725080061</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>1.816964414858432</v>
+        <v>1.8169644147554</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>53.11329216488359</v>
+        <v>53.11329217048142</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.3402772721927</v>
+        <v>29.34027719850388</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.2840684801486197</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-8.974166231488834</v>
+        <v>-8.974166231900949</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>26.91449263061477</v>
+        <v>26.9144925681976</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.28873453848794</v>
+        <v>20.28873457617338</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>2.659930563585315</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-1.068749709720482</v>
+        <v>-1.068749709308368</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>42.73419810786287</v>
+        <v>42.73419802961298</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>6.292490174916185</v>
+        <v>6.292490151203435</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.2969232571657454</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.2435032349516888</v>
+        <v>-0.2435032339419853</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>411.8924853909963</v>
+        <v>411.892485390997</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>33.5</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.4283759746367</v>
+        <v>51.42837598008008</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>11.24981502495758</v>
+        <v>11.24981500705276</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>2.144945046379297</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.8055120904307882</v>
+        <v>-0.8055120905647273</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>25.59109617571812</v>
+        <v>25.59109618031435</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>44.02603372197262</v>
+        <v>44.02603370737011</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.3242453299394727</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-14.09389007150912</v>
+        <v>-14.09389006409302</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>388.2629808033299</v>
+        <v>388.2629808033298</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>66.8</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>53.10248974132215</v>
+        <v>53.10248974333491</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>8.666910111763398</v>
+        <v>8.666910129594429</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>5.269649277363747</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>2.86716401319952</v>
+        <v>2.867164012993461</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3824,7 +3824,7 @@
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>380.2153745824789</v>
+        <v>380.2153745824788</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>62</v>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>53.30098710739651</v>
+        <v>53.30098698975814</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>19.08070905981779</v>
+        <v>19.08070911079731</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.3057990601651973</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.0651954771260328</v>
+        <v>0.0651954772702754</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>56.49992643561865</v>
+        <v>56.4999265231513</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>11.93170695837288</v>
+        <v>11.93170696781978</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.379737219705709</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>46.9226150083757</v>
+        <v>46.92261504340922</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>15.62130375430494</v>
+        <v>15.62130372042743</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.7881617593120971</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.2113237345191824</v>
+        <v>-0.2113237349313137</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>52.2343442618568</v>
+        <v>52.23434422185633</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>14.18375765300733</v>
+        <v>14.18375768546752</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.08490542103636101</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.2877975386578555</v>
+        <v>-0.2877975380396993</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>48.10542930476196</v>
+        <v>48.10542931205821</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>22.38434467860809</v>
+        <v>22.38434468895513</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.8490703580311849</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-2.275228369130445</v>
+        <v>-2.275228369442005</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>28.88422967910678</v>
+        <v>28.8842297165317</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>26.47846214036693</v>
+        <v>26.4784622272068</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.2515688110578468</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.1349527144935884</v>
+        <v>-0.1349527145760096</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>49.70976592499301</v>
+        <v>49.70976616278596</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>18.40986502783893</v>
+        <v>18.40986502480808</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.1064196542416068</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.6026350009305257</v>
+        <v>-0.602635000724472</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>35.86975267006527</v>
+        <v>35.86975260108412</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>30.46527943262149</v>
+        <v>30.46527944390206</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.3478056344090795</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.3480652700677904</v>
+        <v>0.3480652703768605</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>347.805372498968</v>
+        <v>347.8053724989632</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>75.90000000000001</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>47.33953982427768</v>
+        <v>47.33953981455559</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>14.25081776801867</v>
+        <v>14.25081780739634</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>1.081134147129109</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0271414013657091</v>
+        <v>0.0271414016747998</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>47.12838578181336</v>
+        <v>47.12838578476033</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.4420356914128</v>
+        <v>14.44203569772721</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.3835191283189607</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-3.907886026864768</v>
+        <v>-3.907886027070805</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>55.99330842805411</v>
+        <v>55.99330826593896</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>5.439443676096559</v>
+        <v>5.439443577654109</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.0663906409553422</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.3681419381152865</v>
+        <v>0.3681419381771017</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>46.02942548905015</v>
+        <v>46.02942545454994</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>11.34222434643266</v>
+        <v>11.34222433093612</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.10619219299216</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0179792333019042</v>
+        <v>0.0179792332812983</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>34.00252145858759</v>
+        <v>34.00252138176798</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>34.54912933127657</v>
+        <v>34.54912936804278</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.5076744497622739</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>4.607378593065075</v>
+        <v>4.607378594095415</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>51.09215500812525</v>
+        <v>51.09215501977064</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>18.42451725057558</v>
+        <v>18.42451726888373</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.1811487117533486</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-3.689760053050621</v>
+        <v>-3.689760053462715</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>46.21088617631366</v>
+        <v>46.21088630954625</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>33.72927046760945</v>
+        <v>33.72927044186108</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.5805763611930727</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.2050039776648692</v>
+        <v>-0.2050039777885015</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>41.51202723258608</v>
+        <v>41.51202706080401</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>13.36231673563224</v>
+        <v>13.3623166857139</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.2478980212714906</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.0313640179354055</v>
+        <v>-0.0313640170699636</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4714,21 +4714,21 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6955</v>
+        <v>6996</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>邦睿生技-創</t>
+          <t>力領科技</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>307.0368194841387</v>
+        <v>321.1933952318425</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>94.2</v>
+        <v>171</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>49.10209863555261</v>
+        <v>45.39234208774621</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>7.310514395775733</v>
+        <v>16.4257699639824</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.1423727566480474</v>
+        <v>0.1708508601654355</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>1.314715447485255</v>
+        <v>0.0234700955657314</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6862</v>
+        <v>6955</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>邦睿生技-創</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>305.3540150222713</v>
+        <v>307.0368194841384</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>139</v>
+        <v>94.2</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>50.75190703017771</v>
+        <v>49.10209860471768</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>16.4062665823438</v>
+        <v>7.310514408151633</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.3278114144916101</v>
+        <v>0.1423727566480474</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>2</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>1.147797414409259</v>
+        <v>1.314715449133716</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>7791</v>
+        <v>6862</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>304.98671644499</v>
+        <v>305.3540150222713</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>55.8</v>
+        <v>139</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>43.77273150529136</v>
+        <v>50.75190705928935</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>18.84752889449166</v>
+        <v>16.40626660837078</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.3807462954823302</v>
+        <v>0.3278114144916101</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.182766825399493</v>
+        <v>1.147797414306233</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
+          <t>market_above_ma60, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6916</v>
+        <v>7791</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>300.0680581607792</v>
+        <v>304.98671644499</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>18.3</v>
+        <v>55.8</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>47.56062021837991</v>
+        <v>43.77273178876139</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>13.5241848000286</v>
+        <v>18.8475288419396</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.5430523397486822</v>
+        <v>0.3807462954823302</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.008619859790084001</v>
+        <v>0.1827668254613138</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>7721</v>
+        <v>6916</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>294.2325860581765</v>
+        <v>300.0680581607791</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>61.7</v>
+        <v>18.3</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>51.49877639887195</v>
+        <v>47.56062020600491</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>14.76715240700266</v>
+        <v>13.52418480409379</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5632422964452237</v>
+        <v>0.5430523397486822</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.3477027447238744</v>
+        <v>-0.008619859738569401</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4979,21 +4979,21 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6863</v>
+        <v>7721</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>永道-KY</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>293.9740546194832</v>
+        <v>294.2325860581765</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>97.3</v>
+        <v>61.7</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>39.90103530316309</v>
+        <v>51.49877655982996</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>22.76512626628457</v>
+        <v>14.76715235595039</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.5330171917698372</v>
+        <v>0.5632422964452237</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.471595017339137</v>
+        <v>0.3477027442911535</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>7818</v>
+        <v>6863</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>永道-KY</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>285.3091784075782</v>
+        <v>293.9740546194832</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>59.9</v>
+        <v>97.3</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>36.11033789971715</v>
+        <v>39.90103546451419</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>16.58017449869513</v>
+        <v>22.76512623792529</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.4386690823019178</v>
+        <v>0.5330171917698372</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.1502759397784383</v>
+        <v>0.471595016617937</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6967</v>
+        <v>7818</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>285.3089518505918</v>
+        <v>285.3091784075782</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>65.7</v>
+        <v>59.9</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,16 +5110,16 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>38.81021296729335</v>
+        <v>36.11033851770084</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>12.55437640850685</v>
+        <v>16.58017455457361</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.6048393663277402</v>
+        <v>0.4386690823019178</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0039431095294855</v>
+        <v>0.1502759396754058</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6899</v>
+        <v>6967</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>270.4791100106788</v>
+        <v>285.3089518505919</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>49.4</v>
+        <v>65.7</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>42.90299165308684</v>
+        <v>38.81021298295189</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>24.15818297644222</v>
+        <v>12.55437640850685</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5004194692609981</v>
+        <v>0.6048393663277402</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.08065009154643429</v>
+        <v>0.003943109550097</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6952</v>
+        <v>6899</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>大武山</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>270.4598458439602</v>
+        <v>270.4791100106788</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>38.5</v>
+        <v>49.4</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>51.89270313478061</v>
+        <v>42.90299175020188</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>13.7091755664674</v>
+        <v>24.15818294055889</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.1520606113596879</v>
+        <v>0.5004194692609981</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-1.245920687206795</v>
+        <v>0.08065009154643429</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6965</v>
+        <v>6952</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>大武山</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>267.5049370731904</v>
+        <v>270.4598458439604</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>67.09999999999999</v>
+        <v>38.5</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>27.51286756017795</v>
+        <v>51.89270313370801</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>42.52648224305862</v>
+        <v>13.70917558565306</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1.052162727233444</v>
+        <v>0.1520606113596879</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.2428974568199797</v>
+        <v>-1.245920687196486</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>7750</v>
+        <v>6965</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>新代</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>264.0245095890492</v>
+        <v>267.5049370731898</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>1970</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>40.75396604368088</v>
+        <v>27.51286764136665</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>19.43850374729652</v>
+        <v>42.52648221425046</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.5647664245513143</v>
+        <v>1.052162727233444</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-17.89786115820199</v>
+        <v>-0.2428974570260438</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6996</v>
+        <v>7750</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>力領科技</t>
+          <t>新代</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>261.1933952318425</v>
+        <v>264.0245095890493</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>171</v>
+        <v>1970</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>45.39234199401074</v>
+        <v>40.75396605451829</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>16.4257699639824</v>
+        <v>19.43850373898022</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.1708508601654355</v>
+        <v>0.5647664245513143</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,11 +5393,11 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.0234700959778333</v>
+        <v>-17.89786116005699</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>40.10930382415178</v>
+        <v>40.10930386319246</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>19.22481951753726</v>
+        <v>19.22481955455036</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.1529026532559793</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.9219771968081928</v>
+        <v>-0.9219771970142432</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>47.3728227235479</v>
+        <v>47.37282283303127</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>16.91268011822676</v>
+        <v>16.91268011887404</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.571944163086631</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.5027106227717717</v>
+        <v>0.5027106225657203</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>247.5929941941232</v>
+        <v>247.5929941941231</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>45.4</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>39.32085908577142</v>
+        <v>39.32085905851452</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>9.944732028409163</v>
+        <v>9.944732043297526</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.6024097535553077</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.09800412985886831</v>
+        <v>-0.09800412975584</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>243.7240338501623</v>
+        <v>243.7240338501624</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>36</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>52.39496275418066</v>
+        <v>52.39496268808701</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>19.47582618046632</v>
+        <v>19.4758261437482</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.4215546435894839</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.1885446056250705</v>
+        <v>0.1885446055014411</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>27.0555012178753</v>
+        <v>27.05550138419703</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>42.67157280088928</v>
+        <v>42.67157280759388</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4256516148177457</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.8510932681847798</v>
+        <v>0.8510932686999269</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>239.7508992434574</v>
+        <v>239.7508992434575</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>69.2</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>31.72235406631961</v>
+        <v>31.72235395064166</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>32.10013968303346</v>
+        <v>32.1001398178628</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.7649404112327257</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.07794286356242</v>
+        <v>-0.07794286350061411</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>39.64310424604387</v>
+        <v>39.64310431658512</v>
       </c>
       <c r="I101" s="2" t="n">
         <v>17.4841811280855</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.3836635339968678</v>
+        <v>-0.3836635342750444</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,7 +5852,7 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>49.72881662006205</v>
+        <v>49.72881680558567</v>
       </c>
       <c r="I102" s="2" t="n">
         <v>22.06861187863564</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0720969895234327</v>
+        <v>0.0720969895543416</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>229.5177067089404</v>
+        <v>229.5177067089403</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>68.7</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>46.0613417557721</v>
+        <v>46.06134181893098</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>15.00126857357527</v>
+        <v>15.00126860137062</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.6966091070309193</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.0005189862049784</v>
+        <v>0.0005189860813492</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>37.28399122521604</v>
+        <v>37.28399120210859</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>10.25858589205435</v>
+        <v>10.25858592693803</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>1.086577235200064</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.0187523703426574</v>
+        <v>0.0187523703735641</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>212.9805021897155</v>
+        <v>212.9805021897154</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>33</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>49.733619553091</v>
+        <v>49.73362003819879</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>20.0680850746126</v>
+        <v>20.06808507805397</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.9233775751160328</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.0458039574577192</v>
+        <v>0.0458039570971182</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>50.27916820788019</v>
+        <v>50.27916828420292</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>12.99977284272287</v>
+        <v>12.99977284272286</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.137532529639746</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.9156632063289858</v>
+        <v>0.9156632065350374</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>212.0189258795201</v>
+        <v>212.0189258795195</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>157</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>35.21368017737181</v>
+        <v>35.21368028929254</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>18.73159518145819</v>
+        <v>18.73159536659672</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.1342714134995215</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.9844787397047324</v>
+        <v>-0.984478740941082</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>49.97712824842556</v>
+        <v>49.97712846865264</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>14.56838724470968</v>
+        <v>14.568387258024</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.175872429816088</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.1334305252612824</v>
+        <v>0.1334305252715845</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>211.531439674417</v>
+        <v>211.5314396744168</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>29.9</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>43.35764206601068</v>
+        <v>43.35764208658485</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>13.14246720936923</v>
+        <v>13.14246719806754</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.3703006550637505</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0257456101620341</v>
+        <v>0.0257456101826405</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>26.29304481052148</v>
+        <v>26.29304467250913</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>45.88000751389967</v>
+        <v>45.88000755584242</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.341198070319232</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.212671011884332</v>
+        <v>-0.212671011595849</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>37.31321958912049</v>
+        <v>37.31324574650844</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.8043807247171</v>
+        <v>17.80439375816811</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.7248747373525133</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0163257205848847</v>
+        <v>-0.0163257156800621</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>37.06005908317457</v>
+        <v>37.06005919156516</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>31.82408739840109</v>
+        <v>31.82408748719988</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.9822805939556568</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0536191600566262</v>
+        <v>0.0536191600360205</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>40.77600748012584</v>
+        <v>40.77600841203827</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>18.66255189970989</v>
+        <v>18.66255181310962</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.8278194825950294</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.4318415952931691</v>
+        <v>0.4318415935416715</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>38.11756517956725</v>
+        <v>38.11756522866126</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>9.197868771601479</v>
+        <v>9.197868685003217</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.8066911236486998</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.2330417668077431</v>
+        <v>0.2330417668901634</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>41.37153497522229</v>
+        <v>41.37153542378393</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>22.41762486276293</v>
+        <v>22.41762486276294</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.9443578883086584</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.1148950278876161</v>
+        <v>0.1148950273724757</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>27.26687647595003</v>
+        <v>27.26687677447897</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>19.95828183046317</v>
+        <v>19.95828183456467</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.5687485068116084</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.2289040775784171</v>
+        <v>-0.2289040777123527</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>49.93858820004027</v>
+        <v>49.93858815098997</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>18.40936668135708</v>
+        <v>18.40936665019808</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.4916244834366081</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.1686530251108418</v>
+        <v>0.1686530252344774</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>35.10790373644585</v>
+        <v>35.10790376208944</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>15.03040479035827</v>
+        <v>15.03040474843456</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.4443064838542079</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1838191405314447</v>
+        <v>-0.1838191405726628</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>142.1933024789096</v>
+        <v>142.1933024789097</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>145</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>51.56980962247387</v>
+        <v>51.5698096662837</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>19.35802573623702</v>
+        <v>19.35802581061606</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.5439348172731634</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-1.856718101135564</v>
+        <v>-1.85671810041437</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>139.5321418530047</v>
+        <v>139.5321418530048</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>69.8</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>36.9057009941934</v>
+        <v>36.90570103227997</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>14.435798685415</v>
+        <v>14.43579871837796</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.8083101342193236</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.945394652624317</v>
+        <v>-0.9453946525418896</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>42.27898602754767</v>
+        <v>42.27898603115648</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>8.468198599779445</v>
+        <v>8.468198598082136</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.0041648802596925</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>44.72230422900982</v>
+        <v>44.72230427440348</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>14.52039499140345</v>
+        <v>14.52039502271981</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.5918451182354527</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-5.064653211048579</v>
+        <v>-5.064653213624267</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>119.8310822663607</v>
+        <v>119.8310822663604</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>146.5</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>35.27540349654674</v>
+        <v>35.27540359924681</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>11.41009627447381</v>
+        <v>11.41009625503614</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.6016447312122405</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.2248695854810094</v>
+        <v>-0.2248695867173609</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>108.8938365736935</v>
+        <v>108.8938365736936</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>260</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>37.3573219500925</v>
+        <v>37.3573222544471</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>15.24261175473047</v>
+        <v>15.24261175323397</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.8254222631391014</v>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>104.6124029740306</v>
+        <v>104.6124029740316</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>31.7</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>39.76604776948753</v>
+        <v>39.76604798442099</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>19.78636769167145</v>
+        <v>19.78636776225825</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.6525709512737881</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.0633563908695363</v>
+        <v>-0.0633563909828716</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>34.55644238085013</v>
+        <v>34.55644287223868</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>15.52855987900107</v>
+        <v>15.52855985991802</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.2268537890010969</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.0189882175988688</v>
+        <v>0.0189882172897788</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7180,7 +7180,7 @@
         <v>36.07982127144675</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>10.48557687174602</v>
+        <v>10.48557689822373</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.5584866308617499</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.0611868654839983</v>
+        <v>-0.0611868655046041</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>79.41195368245916</v>
+        <v>79.41195368245917</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>91.40000000000001</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>47.12064048285987</v>
+        <v>47.12064058629653</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>14.3356503501744</v>
+        <v>14.33565036922825</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.6275719975104568</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>0.5400255075854863</v>
+        <v>0.5400255070703455</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg7 2026-09-29 00:37 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq8_2026-09-24.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>70.82555094500356</v>
+        <v>70.82555095768525</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>42.70699612569278</v>
+        <v>42.70699612971929</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>3.50021136580328</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.5947603028677833</v>
+        <v>0.5947603026452271</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>65.73815825712292</v>
+        <v>65.73815823578747</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>36.16735081109153</v>
+        <v>36.16735086034097</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.32951480466362</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2.237048119093824</v>
+        <v>2.237048119650156</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>88.12036762146396</v>
+        <v>88.1203676258215</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>52.76802222817642</v>
+        <v>52.76802224173456</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>3.694900644269135</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>9.703150062089811</v>
+        <v>9.703150061978508</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>80.59606979049521</v>
+        <v>80.59606970283258</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>38.51526497614011</v>
+        <v>38.51526500411981</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.79021669540324</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>84.64618590643579</v>
+        <v>84.64618590764087</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>28.18194124558111</v>
+        <v>28.1819411440955</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.964987880141097</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>5.655529836690024</v>
+        <v>5.655529836779039</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>60.24136511461965</v>
+        <v>60.2413651352496</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>29.89846454114974</v>
+        <v>29.89846454304896</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.7287850130249796</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.9773198893429544</v>
+        <v>0.9773198909007448</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61.56154340515053</v>
+        <v>61.56154336111966</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>20.60138748824996</v>
+        <v>20.60138752986498</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.646130978574432</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1.582751406080825</v>
+        <v>1.582751406303362</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>71.15612114256673</v>
+        <v>71.1561211386007</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>27.96381740672689</v>
+        <v>27.96381739220153</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.947854418330473</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>9.354177174787958</v>
+        <v>9.354177174654421</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>875.65480114635</v>
+        <v>875.6548011463499</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>264.5</v>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>61.89811437501302</v>
+        <v>61.89811443889735</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>24.34335075024725</v>
+        <v>24.34335079824757</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.8722209081356974</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.463588909667718</v>
+        <v>1.463588909333934</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>74.94937908256603</v>
+        <v>74.94937910626641</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>15.7037568089477</v>
+        <v>15.70375742081</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>7.431792589963899</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.9119300801061192</v>
+        <v>0.9119300826653584</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>863.4494421920218</v>
+        <v>863.4494421920219</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>304.5</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>61.23935037709227</v>
+        <v>61.23935043030026</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>21.13146529911164</v>
+        <v>21.1314653445356</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.656645262341546</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>4.134038478836409</v>
+        <v>4.134038477946233</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>73.40039407334228</v>
+        <v>73.40039421121813</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>24.66302370393021</v>
+        <v>24.66302361916221</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>6.896318692442442</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.476158059470213</v>
+        <v>1.476158058580047</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.20963148408136</v>
+        <v>60.20963142718386</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>19.50827034222214</v>
+        <v>19.50827034553477</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.96418142760855</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>5.155443507059225</v>
+        <v>5.155443509173388</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>785.9471804295571</v>
+        <v>785.9471804295583</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>760</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>60.57119890552397</v>
+        <v>60.57119888621808</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>19.74367257648731</v>
+        <v>19.74367255005953</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.464175916175535</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>10.06426793670204</v>
+        <v>10.06426793792608</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>766.2575404143539</v>
+        <v>766.2575404143543</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>31.15</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>71.99656052948484</v>
+        <v>71.9965604392106</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>61.5853877572023</v>
+        <v>61.58538783574084</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.151407788814635</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.3573129383142135</v>
+        <v>0.3573129385256328</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>765.9427607578477</v>
+        <v>765.9427607578472</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>920</v>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57.41107416965205</v>
+        <v>57.41107420629328</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>11.03507969234604</v>
+        <v>11.03507969581108</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.928030176784718</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>5.266079005445951</v>
+        <v>5.2660790034431</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>60.96365472454443</v>
+        <v>60.96365474073305</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>16.05187964734687</v>
+        <v>16.05187968262858</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.95934996305407</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.405953840474611</v>
+        <v>1.405953839806988</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>63.90508980610159</v>
+        <v>63.90508966033897</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>17.65705385881593</v>
+        <v>17.65705396088538</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.026247695877518</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>5.059281732021321</v>
+        <v>5.059281735582035</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>58.6925391057643</v>
+        <v>58.69253902878925</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>25.26471035215904</v>
+        <v>25.2647104028884</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.188355694964051</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.9567137103786276</v>
+        <v>0.9567137110462518</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>59.49033415846048</v>
+        <v>59.49033401985781</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>21.08751463240392</v>
+        <v>21.08751460563031</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.131605854810355</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.265345980238305</v>
+        <v>1.265345981239755</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>66.16320063894881</v>
+        <v>66.16320055925343</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>40.57215948541117</v>
+        <v>40.57215951207677</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.4749616713588787</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.3246504560811498</v>
+        <v>0.3246504572828872</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>62.10673352040608</v>
+        <v>62.10673348462745</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>28.88577332024221</v>
+        <v>28.88577322141616</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>1.217587710690275</v>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>658.6835753644948</v>
+        <v>658.6835753644947</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>38.95</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>56.699097918556</v>
+        <v>56.69909801942853</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>36.68749386794412</v>
+        <v>36.68749380147659</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.4801528806772076</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.0943347645566244</v>
+        <v>0.0943347643785897</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>647.8520526270894</v>
+        <v>647.8520526270867</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>26</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>61.46742347205804</v>
+        <v>61.46742361415678</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>26.82029584265646</v>
+        <v>26.82029584827855</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.9874025605664936</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.11866938879235</v>
+        <v>0.1186693886810781</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>65.13566849947772</v>
+        <v>65.13566844645328</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>40.19505521140578</v>
+        <v>40.19505522387926</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>2.095972335302705</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>10.7866561708303</v>
+        <v>10.78665616904998</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>60.68122759345317</v>
+        <v>60.68122761214355</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>36.96136082243196</v>
+        <v>36.96136086665175</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.3678965103766107</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.836592911570146</v>
+        <v>1.836592911236321</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>630.9305996130994</v>
+        <v>630.9305996130993</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>25.5</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>63.58352312051476</v>
+        <v>63.58352291229471</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>27.89889847429074</v>
+        <v>27.89889844589828</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>3.23943968405878</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.201840212163972</v>
+        <v>0.201840212342007</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>621.7126840857229</v>
+        <v>621.7126840857235</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>367</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>58.64700291271885</v>
+        <v>58.64700296340608</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>28.68549034526885</v>
+        <v>28.68549038462964</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.6132911845246226</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.548265763423979</v>
+        <v>1.548265761866169</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>617.5235908407383</v>
+        <v>617.5235908407382</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>121</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>59.77957896588754</v>
+        <v>59.77957882294683</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>39.21054989516679</v>
+        <v>39.21054989717183</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.6433430915393756</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1882100983509431</v>
+        <v>0.188210098796028</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>616.5411665595872</v>
+        <v>616.5411665595871</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>222.5</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>54.87417903911388</v>
+        <v>54.87417893831195</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>31.74107012414833</v>
+        <v>31.74107012238932</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.778876730455374</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.1176190998346982</v>
+        <v>0.1176191010586853</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>49.02213551717188</v>
+        <v>49.02213549519041</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>17.63059829913762</v>
+        <v>17.63059825092652</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.8553368734082714</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>11.04519937159101</v>
+        <v>11.0451993800482</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2251,7 +2251,7 @@
         <v>58.28766715545677</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>34.23908860829906</v>
+        <v>34.23908867805145</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.3851310249883942</v>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>584.9331002489739</v>
+        <v>584.9331002489738</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>348.5</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>55.94041261046966</v>
+        <v>55.94041246614347</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>26.19077985797317</v>
+        <v>26.19077980712354</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.4460736239295284</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-1.09456867925168</v>
+        <v>-1.094568675468503</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>55.90906283543966</v>
+        <v>55.90906281893075</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>42.23952009668248</v>
+        <v>42.23952007196245</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.3749508866699448</v>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>51.58661034996177</v>
+        <v>51.58661035177335</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>15.31131549178912</v>
+        <v>15.3113155054989</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.5051365967127892</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-9.686543585903079</v>
+        <v>-9.686543587572094</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>545.6144112174882</v>
+        <v>545.6144112175025</v>
       </c>
       <c r="E39" s="2" t="n">
         <v>122.5</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>55.46447632677341</v>
+        <v>55.46447633101861</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>17.26019775199913</v>
+        <v>17.26019772924213</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.3806905232054802</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>1.588952145082768</v>
+        <v>1.588952144882475</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>48.46117473868623</v>
+        <v>48.46117471722305</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>21.13086286632531</v>
+        <v>21.13086293843327</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.3571932736127358</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-1.04588927637321</v>
+        <v>-1.045889276128401</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>51.15670335808578</v>
+        <v>51.15670335624318</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>13.99411225358634</v>
+        <v>13.99411224276472</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.577488279054458</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.6485987159527404</v>
+        <v>0.6485987164425708</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>53.82603798567551</v>
+        <v>53.82603798278853</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>25.40657876632234</v>
+        <v>25.4065786361576</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.3946859086876488</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-3.766801086328769</v>
+        <v>-3.766801084326005</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>43.11357763512334</v>
+        <v>43.11358511465238</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>35.78384472633256</v>
+        <v>35.78384310521079</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1.506827072108643</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0196544880597784</v>
+        <v>0.0196544727043322</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>49.713669631964</v>
+        <v>49.71366961590842</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>13.07216748591079</v>
+        <v>13.07216748102985</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.8008435049063258</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>1.856836412218478</v>
+        <v>1.856836412329768</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>59.10791685129321</v>
+        <v>59.10791658488814</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>20.90060718451973</v>
+        <v>20.90060726777827</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.8831122832831965</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.7626195154181873</v>
+        <v>0.7626195160858233</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>49.85256269669333</v>
+        <v>49.85256245984154</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>10.04010459683971</v>
+        <v>10.04010470727302</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.3491499896645576</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.1252319418196713</v>
+        <v>0.1252319419420696</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>443.698134337455</v>
+        <v>443.6981343374548</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>5670</v>
@@ -3096,7 +3096,7 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>40.192844213586</v>
+        <v>40.19284421985304</v>
       </c>
       <c r="I50" s="2" t="n">
         <v>11.65234407452498</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-52.74734770305497</v>
+        <v>-52.74734770082948</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3152,7 +3152,7 @@
         <v>56.78614114756991</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>23.1412094684832</v>
+        <v>23.14120950979536</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.9701417725852</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.072679934387053</v>
+        <v>0.0726799344093059</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>45.55765966704588</v>
+        <v>45.55765963280635</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>25.97607906387721</v>
+        <v>25.97607903024112</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6506872437906921</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0157128620253457</v>
+        <v>0.0157128620587249</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>53.05379800273698</v>
+        <v>53.05379799879101</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>18.68221079673399</v>
+        <v>18.68221080628512</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.068079424069768</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.033076917601218</v>
+        <v>-0.0330769175789607</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>47.6381929455761</v>
+        <v>47.63819297614106</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>11.54075631245025</v>
+        <v>11.54075631866167</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.6138697630524275</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.5955569773648346</v>
+        <v>0.5955569774761189</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>51.28007099387669</v>
+        <v>51.28007085374147</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.66629194508466</v>
+        <v>18.66629179264464</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.1007261379169665</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.5991054042578497</v>
+        <v>-0.5991054039240368</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>51.65881442467627</v>
+        <v>51.65881442813722</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>7.417385959696069</v>
+        <v>7.417385968407339</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.2942788725080061</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>1.8169644147554</v>
+        <v>1.81696441464412</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>53.11329217048142</v>
+        <v>53.1132921681569</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.34027719850388</v>
+        <v>29.34027734040054</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.2840684801486197</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-8.974166231900949</v>
+        <v>-8.974166231789717</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>26.9144925681976</v>
+        <v>26.91449253910264</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.28873457617338</v>
+        <v>20.28873465763598</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>2.659930563585315</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-1.068749709308368</v>
+        <v>-1.068749709642166</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>42.73419802961298</v>
+        <v>42.73419818439299</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>6.292490151203435</v>
+        <v>6.292490177881287</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.2969232571657454</v>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>411.892485390997</v>
+        <v>411.8924853909966</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>33.5</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.42837598008008</v>
+        <v>51.42837598140003</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>11.24981500705276</v>
+        <v>11.24981505455112</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>2.144945046379297</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.8055120905647273</v>
+        <v>-0.805512090520218</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>25.59109618031435</v>
+        <v>25.59109618650159</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>44.02603370737011</v>
+        <v>44.02603373267467</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.3242453299394727</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-14.09389006409302</v>
+        <v>-14.09389005532091</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>388.2629808033298</v>
+        <v>388.2629808033303</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>66.8</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>53.10248974333491</v>
+        <v>53.1024897121218</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>8.666910129594429</v>
+        <v>8.666910138909506</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>5.269649277363747</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>2.867164012993461</v>
+        <v>2.867164012882183</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,7 +3838,7 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>53.30098698975814</v>
+        <v>53.30098704354196</v>
       </c>
       <c r="I64" s="2" t="n">
         <v>19.08070911079731</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.0651954772702754</v>
+        <v>0.0651954770922355</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>372.4913775208336</v>
+        <v>372.4913775208335</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>28.05</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>56.4999265231513</v>
+        <v>56.4999264726517</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>11.93170696781978</v>
+        <v>11.93170711942139</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.379737219705709</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.0729184212368387</v>
+        <v>0.07291842185995941</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,7 +3944,7 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>46.92261504340922</v>
+        <v>46.92261499310467</v>
       </c>
       <c r="I66" s="2" t="n">
         <v>15.62130372042743</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.2113237349313137</v>
+        <v>-0.2113237350425847</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,7 +3997,7 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>52.23434422185633</v>
+        <v>52.23434424064272</v>
       </c>
       <c r="I67" s="2" t="n">
         <v>14.18375768546752</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.2877975380396993</v>
+        <v>-0.2877975381509579</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>48.10542931205821</v>
+        <v>48.10542931991573</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>22.38434468895513</v>
+        <v>22.38434471199184</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.8490703580311849</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-2.275228369442005</v>
+        <v>-2.275228369610248</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>28.8842297165317</v>
+        <v>28.88422978040673</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>26.4784622272068</v>
+        <v>26.47846215315011</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.2515688110578468</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.1349527145760096</v>
+        <v>-0.1349527146093894</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>356.6722833390184</v>
+        <v>356.6722833390185</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>172</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>49.70976616278596</v>
+        <v>49.70976592998167</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>18.40986502480808</v>
+        <v>18.40986525258995</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.1064196542416068</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.602635000724472</v>
+        <v>-0.6026349968299739</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>35.86975260108412</v>
+        <v>35.86975264361105</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>30.46527944390206</v>
+        <v>30.46527944567378</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.3478056344090795</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.3480652703768605</v>
+        <v>0.3480652700430511</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>347.8053724989632</v>
+        <v>347.8053724989502</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>75.90000000000001</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>47.33953981455559</v>
+        <v>47.33953903737049</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>14.25081780739634</v>
+        <v>14.25081789474513</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>1.081134147129109</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0271414016747998</v>
+        <v>0.0271414019863618</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>47.12838578476033</v>
+        <v>47.12838579544153</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.44203569772721</v>
+        <v>14.44203570524206</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.3835191283189607</v>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>340.4228440925754</v>
+        <v>340.4228440925757</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>39.5</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>55.99330826593896</v>
+        <v>55.99330842818452</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>5.439443577654109</v>
+        <v>5.439443555613508</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.0663906409553422</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.3681419381771017</v>
+        <v>0.368141937487221</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>46.02942545454994</v>
+        <v>46.0294255040887</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>11.34222433093612</v>
+        <v>11.34222442554912</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.10619219299216</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0179792332812983</v>
+        <v>0.0179792332256619</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>34.00252138176798</v>
+        <v>34.0025214260472</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>34.54912936804278</v>
+        <v>34.54912936180828</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.5076744497622739</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>4.607378594095415</v>
+        <v>4.607378592537632</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4583,7 +4583,7 @@
         <v>51.09215501977064</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>18.42451726888373</v>
+        <v>18.42451724348753</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.1811487117533486</v>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>327.4147850287659</v>
+        <v>327.414785028766</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>74.2</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>46.21088630954625</v>
+        <v>46.2108861736954</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>33.72927044186108</v>
+        <v>33.72927048600165</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.5805763611930727</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.2050039777885015</v>
+        <v>-0.2050039775437137</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>41.51202706080401</v>
+        <v>41.5120270125507</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>13.3623166857139</v>
+        <v>13.36231673963016</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.2478980212714906</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.0313640170699636</v>
+        <v>-0.031364017203499</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4714,21 +4714,21 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6996</v>
+        <v>6955</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>力領科技</t>
+          <t>邦睿生技-創</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>321.1933952318425</v>
+        <v>307.0368194841384</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>171</v>
+        <v>94.2</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>45.39234208774621</v>
+        <v>49.10209860234576</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>16.4257699639824</v>
+        <v>7.310514412073495</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.1708508601654355</v>
+        <v>0.1423727566480474</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.0234700955657314</v>
+        <v>1.314715449356262</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6955</v>
+        <v>6862</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>邦睿生技-創</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>307.0368194841384</v>
+        <v>305.3540150222711</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>94.2</v>
+        <v>139</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>49.10209860471768</v>
+        <v>50.75190697463371</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>7.310514408151633</v>
+        <v>16.40626661959971</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.1423727566480474</v>
+        <v>0.3278114144916101</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>2</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>1.314715449133716</v>
+        <v>1.147797414528765</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6862</v>
+        <v>7791</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>305.3540150222713</v>
+        <v>304.98671644499</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>139</v>
+        <v>55.8</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>50.75190705928935</v>
+        <v>43.77273183696276</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>16.40626660837078</v>
+        <v>18.8475293354145</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.3278114144916101</v>
+        <v>0.3807462954823302</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>1.147797414306233</v>
+        <v>0.1827668259509089</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>7791</v>
+        <v>6916</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>304.98671644499</v>
+        <v>300.0680581607791</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>55.8</v>
+        <v>18.3</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>43.77273178876139</v>
+        <v>47.56062014061019</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>18.8475288419396</v>
+        <v>13.52418481343883</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.3807462954823302</v>
+        <v>0.5430523397486822</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.1827668254613138</v>
+        <v>-0.008619859694060501</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6916</v>
+        <v>7721</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>300.0680581607791</v>
+        <v>294.2325860581765</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>18.3</v>
+        <v>61.7</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>47.56062020600491</v>
+        <v>51.49877644302953</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>13.52418480409379</v>
+        <v>14.76715244806008</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5430523397486822</v>
+        <v>0.5632422964452237</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.008619859738569401</v>
+        <v>0.3477027444469313</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4979,21 +4979,21 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>7721</v>
+        <v>6863</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>永道-KY</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>294.2325860581765</v>
+        <v>293.9740546194832</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>61.7</v>
+        <v>97.3</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>51.49877655982996</v>
+        <v>39.901035357456</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>14.76715235595039</v>
+        <v>22.76512637184294</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.5632422964452237</v>
+        <v>0.5330171917698372</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.3477027442911535</v>
+        <v>0.4715950170630112</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6863</v>
+        <v>7818</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>永道-KY</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>293.9740546194832</v>
+        <v>285.3091784075782</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>97.3</v>
+        <v>59.9</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>39.90103546451419</v>
+        <v>36.11033785217995</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>22.76512623792529</v>
+        <v>16.5801750730339</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.5330171917698372</v>
+        <v>0.4386690823019178</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.471595016617937</v>
+        <v>0.1502759402317679</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>7818</v>
+        <v>6967</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>285.3091784075782</v>
+        <v>285.3089518505919</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>59.9</v>
+        <v>65.7</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,16 +5110,16 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>36.11033851770084</v>
+        <v>38.81021295230956</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>16.58017455457361</v>
+        <v>12.55437641433177</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.4386690823019178</v>
+        <v>0.6048393663277402</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.1502759396754058</v>
+        <v>0.0039431096168613</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6967</v>
+        <v>6899</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>285.3089518505919</v>
+        <v>270.4791100106788</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>65.7</v>
+        <v>49.4</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>38.81021298295189</v>
+        <v>42.90299168047827</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>12.55437640850685</v>
+        <v>24.15818298362035</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.6048393663277402</v>
+        <v>0.5004194692609981</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.003943109550097</v>
+        <v>0.08065009167996801</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6899</v>
+        <v>6952</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>大武山</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>270.4791100106788</v>
+        <v>270.4598458439603</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>49.4</v>
+        <v>38.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>42.90299175020188</v>
+        <v>51.89270313094561</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>24.15818294055889</v>
+        <v>13.70917556013714</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.5004194692609981</v>
+        <v>0.1520606113596879</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.08065009154643429</v>
+        <v>-1.245920687218744</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6952</v>
+        <v>6965</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>大武山</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>270.4598458439604</v>
+        <v>267.5049370731899</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>38.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>51.89270313370801</v>
+        <v>27.51286759166312</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>13.70917558565306</v>
+        <v>42.52648230310203</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.1520606113596879</v>
+        <v>1.052162727233444</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-1.245920687196486</v>
+        <v>-0.2428974569147763</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6965</v>
+        <v>7750</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>新代</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>267.5049370731898</v>
+        <v>264.0245095890492</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>67.09999999999999</v>
+        <v>1970</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>27.51286764136665</v>
+        <v>40.75396604678616</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>42.52648221425046</v>
+        <v>19.43850374641953</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>1.052162727233444</v>
+        <v>0.5647664245513143</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.2428974570260438</v>
+        <v>-17.89786115916635</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>7750</v>
+        <v>6996</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>新代</t>
+          <t>力領科技</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>264.0245095890493</v>
+        <v>261.1933952318425</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>1970</v>
+        <v>171</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>40.75396605451829</v>
+        <v>45.39234196388946</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>19.43850373898022</v>
+        <v>16.4257699639824</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.5647664245513143</v>
+        <v>0.1708508601654355</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,11 +5393,11 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-17.89786116005699</v>
+        <v>0.0234700960108114</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>40.10930386319246</v>
+        <v>40.10930381271693</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>19.22481955455036</v>
+        <v>19.22481958473724</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.1529026532559793</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.9219771970142432</v>
+        <v>-0.921977196791679</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>248.1201448153304</v>
+        <v>248.1201448153305</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>118</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>47.37282283303127</v>
+        <v>47.37282295499546</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>16.91268011887404</v>
+        <v>16.91268017964893</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.571944163086631</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.5027106225657203</v>
+        <v>0.5027106230108125</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>39.32085905851452</v>
+        <v>39.32085907808357</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>9.944732043297526</v>
+        <v>9.944732044216224</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.6024097535553077</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.09800412975584</v>
+        <v>-0.0980041297113293</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>52.39496268808701</v>
+        <v>52.39496262580646</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>19.4758261437482</v>
+        <v>19.47582616498257</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.4215546435894839</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.1885446055014411</v>
+        <v>0.1885446052788988</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>27.05550138419703</v>
+        <v>27.05550111552348</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>42.67157280759388</v>
+        <v>42.67157280125137</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4256516148177457</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.8510932686999269</v>
+        <v>0.8510932697013676</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>239.7508992434575</v>
+        <v>239.7508992434574</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>69.2</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>31.72235395064166</v>
+        <v>31.72235433163036</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>32.1001398178628</v>
+        <v>32.10013984711073</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.7649404112327257</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.07794286350061411</v>
+        <v>-0.07794286358963159</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>39.64310431658512</v>
+        <v>39.64310424061762</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>17.4841811280855</v>
+        <v>17.48418113348198</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>1.623531285727725</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.3836635342750444</v>
+        <v>-0.3836635342639205</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>49.72881680558567</v>
+        <v>49.72881666726629</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>22.06861187863564</v>
+        <v>22.06861205338156</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.4188297036523866</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0720969895543416</v>
+        <v>0.0720969897323748</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>229.5177067089403</v>
+        <v>229.5177067089402</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>68.7</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>46.06134181893098</v>
+        <v>46.06134180782386</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>15.00126860137062</v>
+        <v>15.00126877906194</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.6966091070309193</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.0005189860813492</v>
+        <v>0.0005189861035906</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>37.28399120210859</v>
+        <v>37.28399182423246</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>10.25858592693803</v>
+        <v>10.25858599006781</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>1.086577235200064</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.0187523703735641</v>
+        <v>0.0187523703958186</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>212.9805021897154</v>
+        <v>212.9805021897155</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>33</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>49.73362003819879</v>
+        <v>49.73361950514585</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>20.06808507805397</v>
+        <v>20.06808506653886</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.9233775751160328</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.0458039570971182</v>
+        <v>0.045803957252902</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>212.2907180657628</v>
+        <v>212.2907180657629</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>108</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>50.27916828420292</v>
+        <v>50.27916816185101</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>12.99977284272286</v>
+        <v>12.99977327734617</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.137532529639746</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.9156632065350374</v>
+        <v>0.915663210207</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>212.0189258795195</v>
+        <v>212.0189258795212</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>157</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>35.21368028929254</v>
+        <v>35.21368038088681</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>18.73159536659672</v>
+        <v>18.73159541018796</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.1342714134995215</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.984478740941082</v>
+        <v>-0.984478741052362</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>49.97712846865264</v>
+        <v>49.97712810735763</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>14.568387258024</v>
+        <v>14.56838754629979</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>1.175872429816088</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.1334305252715845</v>
+        <v>0.1334305255163824</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>211.5314396744168</v>
+        <v>211.531439674417</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>29.9</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>43.35764208658485</v>
+        <v>43.35764171483063</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>13.14246719806754</v>
+        <v>13.14246724335572</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.3703006550637505</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0257456101826405</v>
+        <v>0.0257456102160187</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>26.29304467250913</v>
+        <v>26.2930447255908</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>45.88000755584242</v>
+        <v>45.88000754458951</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.341198070319232</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>37.31324574650844</v>
+        <v>37.31319975553939</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.80439375816811</v>
+        <v>17.80442413244033</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.7248747373525133</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0163257156800621</v>
+        <v>-0.0163256980227014</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>37.06005919156516</v>
+        <v>37.06005907936532</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>31.82408748719988</v>
+        <v>31.8240875770108</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.9822805939556568</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0536191600360205</v>
+        <v>0.0536191601917974</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>40.77600841203827</v>
+        <v>40.77600806064638</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>18.66255181310962</v>
+        <v>18.66255159850305</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.8278194825950294</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.4318415935416715</v>
+        <v>0.4318415950994634</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>38.11756522866126</v>
+        <v>38.11756511883278</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>9.197868685003217</v>
+        <v>9.197868672844606</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.8066911236486998</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.2330417668901634</v>
+        <v>0.2330417671127032</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>41.37153542378393</v>
+        <v>41.3715357139621</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>22.41762486276294</v>
+        <v>22.41762492668808</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.9443578883086584</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.1148950273724757</v>
+        <v>0.1148950274614896</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>27.26687677447897</v>
+        <v>27.26687650487379</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>19.95828183456467</v>
+        <v>19.95828187490949</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.5687485068116084</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.2289040777123527</v>
+        <v>-0.2289040774564239</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>148.6496010610372</v>
+        <v>148.6496010610373</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>41.5</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>49.93858815098997</v>
+        <v>49.9385882214298</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>18.40936665019808</v>
+        <v>18.40936669766764</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.4916244834366081</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.1686530252344774</v>
+        <v>0.168653025201101</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>35.10790376208944</v>
+        <v>35.10790373447327</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>15.03040474843456</v>
+        <v>15.03040475311909</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.4443064838542079</v>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>142.1933024789097</v>
+        <v>142.1933024789095</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>145</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>51.5698096662837</v>
+        <v>51.56980950281373</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>19.35802581061606</v>
+        <v>19.35802591222241</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.5439348172731634</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-1.85671810041437</v>
+        <v>-1.856718099079089</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>36.90570103227997</v>
+        <v>36.90570097245799</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>14.43579871837796</v>
+        <v>14.43579867254398</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.8083101342193236</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.9453946525418896</v>
+        <v>-0.945394652230328</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>42.27898603115648</v>
+        <v>42.27898602499271</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>8.468198598082136</v>
+        <v>8.468198594288982</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.0041648802596925</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-3.643564679631303</v>
+        <v>-3.643564679074936</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,7 +6912,7 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>44.72230427440348</v>
+        <v>44.7223043796638</v>
       </c>
       <c r="I122" s="2" t="n">
         <v>14.52039502271981</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-5.064653213624267</v>
+        <v>-5.064653213735556</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>119.8310822663604</v>
+        <v>119.8310822663606</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>146.5</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>35.27540359924681</v>
+        <v>35.27540348158851</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>11.41009625503614</v>
+        <v>11.41009630430739</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.6016447312122405</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.2248695867173609</v>
+        <v>-0.2248695864948251</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>108.8938365736936</v>
+        <v>108.8938365736935</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>260</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>37.3573222544471</v>
+        <v>37.35732190224741</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>15.24261175323397</v>
+        <v>15.24261203114212</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.8254222631391014</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.3712905931870738</v>
+        <v>-0.3712905896263869</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>39.76604798442099</v>
+        <v>39.76604783436662</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>19.78636776225825</v>
+        <v>19.78636766488664</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.6525709512737881</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.0633563909828716</v>
+        <v>-0.0633563909383638</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>34.55644287223868</v>
+        <v>34.55644253004495</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>15.52855985991802</v>
+        <v>15.52855984988911</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.2268537890010969</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>0.0189882172897788</v>
+        <v>0.0189882175790909</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7180,7 +7180,7 @@
         <v>36.07982127144675</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>10.48557689822373</v>
+        <v>10.48557697722965</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.5584866308617499</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.0611868655046041</v>
+        <v>-0.0611868655268564</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>79.41195368245917</v>
+        <v>79.41195368245916</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>91.40000000000001</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>47.12064058629653</v>
+        <v>47.12064045952678</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>14.33565036922825</v>
+        <v>14.33565040393651</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.6275719975104568</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>0.5400255070703455</v>
+        <v>0.5400255072928812</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>

</xml_diff>